<commit_message>
Committing search employee module tests
</commit_message>
<xml_diff>
--- a/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
+++ b/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bec74d40107829ab/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D69C64-66EE-4BA9-9EFD-C95716E657BA}"/>
+  <xr:revisionPtr revIDLastSave="136" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F15CD0C-6DFC-487B-891B-581428BDD0CC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Logout" sheetId="2" r:id="rId2"/>
     <sheet name="AddEmployee" sheetId="3" r:id="rId3"/>
+    <sheet name="SearchEmployee" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="59">
   <si>
     <t>Username</t>
   </si>
@@ -131,16 +132,108 @@
   </si>
   <si>
     <t>LoginPassword</t>
+  </si>
+  <si>
+    <t>EmpName</t>
+  </si>
+  <si>
+    <t>EmpStatus</t>
+  </si>
+  <si>
+    <t>TC15</t>
+  </si>
+  <si>
+    <t>TC16</t>
+  </si>
+  <si>
+    <t>TC17</t>
+  </si>
+  <si>
+    <t>TC18</t>
+  </si>
+  <si>
+    <t>TC19</t>
+  </si>
+  <si>
+    <t>TC20</t>
+  </si>
+  <si>
+    <t>TC21</t>
+  </si>
+  <si>
+    <t>TC22</t>
+  </si>
+  <si>
+    <t>TC23</t>
+  </si>
+  <si>
+    <t>TC24</t>
+  </si>
+  <si>
+    <t>0042</t>
+  </si>
+  <si>
+    <t>JobTitle</t>
+  </si>
+  <si>
+    <t>Ranga Akunuri</t>
+  </si>
+  <si>
+    <t>Part-Time Contract</t>
+  </si>
+  <si>
+    <t>asdldkjfk@#$</t>
+  </si>
+  <si>
+    <t>564asdf</t>
+  </si>
+  <si>
+    <t>SupervisorName</t>
+  </si>
+  <si>
+    <t>1024</t>
+  </si>
+  <si>
+    <t>Full-Time Contract</t>
+  </si>
+  <si>
+    <t>2643</t>
+  </si>
+  <si>
+    <t>492</t>
+  </si>
+  <si>
+    <t>1182</t>
+  </si>
+  <si>
+    <t>Fernandes</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Fernandes Gabriel</t>
+  </si>
+  <si>
+    <t>Automaton Tester</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -163,14 +256,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -764,4 +860,240 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4672A6-5E3B-4378-A53C-9FAD69B2BAA6}">
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F8" r:id="rId1" xr:uid="{B5C527E8-CD81-4C18-AD7D-75F5B8119F9E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
committing Update employee tests
</commit_message>
<xml_diff>
--- a/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
+++ b/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bec74d40107829ab/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="136" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F15CD0C-6DFC-487B-891B-581428BDD0CC}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33F34819-56C9-4F5A-A66A-7C8B80D6BD39}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Logout" sheetId="2" r:id="rId2"/>
     <sheet name="AddEmployee" sheetId="3" r:id="rId3"/>
     <sheet name="SearchEmployee" sheetId="4" r:id="rId4"/>
+    <sheet name="UpdateEmployee" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="72">
   <si>
     <t>Username</t>
   </si>
@@ -216,6 +217,45 @@
   </si>
   <si>
     <t>Automaton Tester</t>
+  </si>
+  <si>
+    <t>TC25</t>
+  </si>
+  <si>
+    <t>0320</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>TC26</t>
+  </si>
+  <si>
+    <t>TC27</t>
+  </si>
+  <si>
+    <t>0312</t>
+  </si>
+  <si>
+    <t>UpdateEmpId</t>
+  </si>
+  <si>
+    <t>TC28</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Chief Financial Officer</t>
+  </si>
+  <si>
+    <t>TC29</t>
+  </si>
+  <si>
+    <t>TC30</t>
+  </si>
+  <si>
+    <t>TC31</t>
   </si>
 </sst>
 </file>
@@ -1096,4 +1136,204 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50907181-2A0A-4287-B3BA-F19CBC3C4AD7}">
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="1">
+        <v>8220</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D19" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>